<commit_message>
n8n board refresh 2026-06-20T17:47:00Z
</commit_message>
<xml_diff>
--- a/app/reports/ESSI_research.xlsx
+++ b/app/reports/ESSI_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-19 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-20 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
-        <v>-8.720000000000001</v>
+        <v>-9.81</v>
       </c>
       <c r="F6" s="33" t="n"/>
     </row>
@@ -1537,10 +1537,10 @@
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
-        <v>-1.306</v>
+        <v>-0.902</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>0.371</v>
+        <v>0.257</v>
       </c>
     </row>
     <row r="8">
@@ -1623,10 +1623,10 @@
       </c>
       <c r="D11" s="33" t="n"/>
       <c r="E11" s="33" t="n">
-        <v>-0.854</v>
+        <v>-0.843</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>19.739</v>
+        <v>19.499</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-21T17:48:44Z
</commit_message>
<xml_diff>
--- a/app/reports/ESSI_research.xlsx
+++ b/app/reports/ESSI_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-20 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-21 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.044509997</v>
+        <v>0.04450999999999999</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-22T17:47:26Z
</commit_message>
<xml_diff>
--- a/app/reports/ESSI_research.xlsx
+++ b/app/reports/ESSI_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-21 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-22 17:39 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0.175</v>
+        <v>0.25</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04450999999999999</v>
+        <v>0.04508999824523926</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>24952651.42857143</v>
+        <v>24952656</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>0.175</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="38">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>4366714</v>
+        <v>6238164</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>0</v>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>650264</v>
+        <v>346336</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>20000</v>
+        <v>16000</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n"/>

</xml_diff>

<commit_message>
n8n board refresh 2026-06-23T17:39:30Z
</commit_message>
<xml_diff>
--- a/app/reports/ESSI_research.xlsx
+++ b/app/reports/ESSI_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-22 17:39 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-23 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04508999824523926</v>
+        <v>0.04484999656677246</v>
       </c>
     </row>
     <row r="6">
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>346336</v>
+        <v>650264</v>
       </c>
       <c r="D6" s="33" t="n"/>
       <c r="E6" s="33" t="n">
@@ -1533,14 +1533,14 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>1655951</v>
+        <v>4471068</v>
       </c>
       <c r="D7" s="33" t="n"/>
       <c r="E7" s="33" t="n">
-        <v>-0.902</v>
+        <v>-1.541</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>0.257</v>
+        <v>0.438</v>
       </c>
     </row>
     <row r="8">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>16000</v>
+        <v>20000</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n"/>
@@ -1623,10 +1623,10 @@
       </c>
       <c r="D11" s="33" t="n"/>
       <c r="E11" s="33" t="n">
-        <v>-0.843</v>
+        <v>-0.926</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>19.499</v>
+        <v>21.407</v>
       </c>
     </row>
     <row r="12">

</xml_diff>